<commit_message>
Updating analytical prompt, generating final batch for Hugo
</commit_message>
<xml_diff>
--- a/questions_v3v2_June03.xlsx
+++ b/questions_v3v2_June03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/j_berenguer_cgiar_org/Documents/Microsoft Teams Chat Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlbkm\Coding\document-tagging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42B4F36B-AF1F-44BA-A601-DCF59BDA6E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8934480-DBF7-4CF7-92F4-4CEE40021D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1000" yWindow="1750" windowWidth="29520" windowHeight="15550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q_FOR_SCRIPT" sheetId="1" r:id="rId1"/>
@@ -845,9 +845,75 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:** Impact/Outcome Indicators
+      </rPr>
+      <t>:** Link or DOI.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Description</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Extract the DOI or URL that references to this article in its content.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Output Format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Your response should be a string with the URL.</t>
+    </r>
+  </si>
+  <si>
+    <t>**Parameter:** Crop/Product Type.
+**Description:** Identify CGIAR research object. It could be a crop (e.g. cereals, legumes, fruits, and vegetables), livestock (e.g. cattle, poultry, fish, other animal species) or even an technology innovation. For crop your answer should be based on the vocabulary used in AGROVOC. It possible that CGIAR research is not link to a specific crop or livestock, when this is the case you should reply with "Not specific". And if you identifiy that CGIAR research object is a technology you should reply "technology".
+**Output Format:** Your response should be a string with the values separated by commas. Use your judgement and AGROVOC vocabulary for the response wording.</t>
+  </si>
+  <si>
+    <r>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:** Impact/Outcome Indicators Simple
 **</t>
     </r>
     <r>
@@ -917,78 +983,12 @@
 - Example: `[[""Maize Yield"", ""%"", ""5% increase (p&lt;0.05)""], [""Adoption Rate"", ""Households"", ""20% adoption (p&lt;0.01)""]]`</t>
     </r>
   </si>
-  <si>
-    <r>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Parameter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Link or DOI.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Description</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Extract the DOI or URL that references to this article in its content.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Output Format</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Your response should be a string with the URL.</t>
-    </r>
-  </si>
-  <si>
-    <t>**Parameter:** Crop/Product Type.
-**Description:** Identify CGIAR research object. It could be a crop (e.g. cereals, legumes, fruits, and vegetables), livestock (e.g. cattle, poultry, fish, other animal species) or even an technology innovation. For crop your answer should be based on the vocabulary used in AGROVOC. It possible that CGIAR research is not link to a specific crop or livestock, when this is the case you should reply with "Not specific". And if you identifiy that CGIAR research object is a technology you should reply "technology".
-**Output Format:** Your response should be a string with the values separated by commas. Use your judgement and AGROVOC vocabulary for the response wording.</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1316,16 +1316,16 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="21.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" customWidth="1"/>
-    <col min="8" max="9" width="21.5703125" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" customWidth="1"/>
+    <col min="1" max="2" width="21.59765625" customWidth="1"/>
+    <col min="5" max="5" width="21.59765625" customWidth="1"/>
+    <col min="7" max="7" width="71.59765625" customWidth="1"/>
+    <col min="8" max="9" width="21.59765625" customWidth="1"/>
+    <col min="15" max="15" width="21.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="338.25" customHeight="1">
+    <row r="1" spans="1:15" ht="338.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1366,10 +1366,10 @@
         <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1380,14 +1380,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E6D4E2-1D8F-48EE-9FAC-0B644E8606E1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.95"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="89.85546875" customWidth="1"/>
+    <col min="1" max="1" width="89.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="104.1">
+    <row r="1" spans="1:1" ht="104" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final version with single row output and intermediate outputs, sent 10 to Hugo for final green light review
</commit_message>
<xml_diff>
--- a/questions_v3v2_June03.xlsx
+++ b/questions_v3v2_June03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlbkm\Coding\document-tagging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8934480-DBF7-4CF7-92F4-4CEE40021D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D693D602-3F51-4CF7-87B5-64A5057760BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1000" yWindow="1750" windowWidth="29520" windowHeight="15550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5100" yWindow="5330" windowWidth="29520" windowHeight="15550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q_FOR_SCRIPT" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <r>
       <rPr>
@@ -892,103 +892,12 @@
 **Description:** Identify CGIAR research object. It could be a crop (e.g. cereals, legumes, fruits, and vegetables), livestock (e.g. cattle, poultry, fish, other animal species) or even an technology innovation. For crop your answer should be based on the vocabulary used in AGROVOC. It possible that CGIAR research is not link to a specific crop or livestock, when this is the case you should reply with "Not specific". And if you identifiy that CGIAR research object is a technology you should reply "technology".
 **Output Format:** Your response should be a string with the values separated by commas. Use your judgement and AGROVOC vocabulary for the response wording.</t>
   </si>
-  <si>
-    <r>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Parameter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:** Impact/Outcome Indicators Simple
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Description</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">:** Identify mentions in the text of 
-1) Indicators used to assess the impact/outcome of CGIAR interventions,
-2) Units used to measure results, 
-3) The quantitative or qualitative results of the intervention. 
-Only capture these triplets if the numeric results are reported as statistically significant in the text. If multiple triplets are mentioned, output each as a list of three elements. For other significant or notable results (both quantitative or qualitative information that seems significant or relevant, although technically not statistically significant or not explicitly mentioned) capture them as a separate set of triples [Indicator, Units, Results]. </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>You should start your analysis by screening the sections "Abstract" or "Conclusion" (or similar sections) and based on the findings  you could extend the search to other sections from the study to complete your search.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Output Format</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:** 
-- Return a list of lists, with each nested list containing exactly three items in the order: [Indicator, Units, Results].
-- Separate each nested list with a comma. 
-- If no valid triplets are found, return an empty list.
-- Example: `[[""Maize Yield"", ""%"", ""5% increase (p&lt;0.05)""], [""Adoption Rate"", ""Households"", ""20% adoption (p&lt;0.01)""]]`</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1035,13 +944,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1315,17 +1217,17 @@
     <tabColor rgb="FFF1C232"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="21.59765625" customWidth="1"/>
     <col min="5" max="5" width="21.59765625" customWidth="1"/>
     <col min="7" max="7" width="71.59765625" customWidth="1"/>
     <col min="8" max="9" width="21.59765625" customWidth="1"/>
-    <col min="15" max="15" width="21.59765625" customWidth="1"/>
+    <col min="14" max="14" width="21.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="338.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="338.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1366,9 +1268,6 @@
         <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating code, noticed missing rows on analytical answer
</commit_message>
<xml_diff>
--- a/questions_v3v2_June03.xlsx
+++ b/questions_v3v2_June03.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28926"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlbkm\Coding\document-tagging\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/j_berenguer_cgiar_org/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D693D602-3F51-4CF7-87B5-64A5057760BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F29851E9-F173-41FE-9B62-1FE3446C7755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5100" yWindow="5330" windowWidth="29520" windowHeight="15550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q_FOR_SCRIPT" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Analytical Prompt" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <r>
       <rPr>
@@ -295,22 +296,26 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
       <t>**</t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>Parameter</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>:** Contributing Initiatives or centers.
@@ -320,37 +325,116 @@
       <rPr>
         <b/>
         <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>Description</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">:** CGIAR is associated with multiple Initiatives and Centers. You need to extract the names of the ones mentioned in the text, if any.
-**Output Format:** Your response should be a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>string with values separated by commas</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>. For example "CIMMYT, AgriLac Resiliente, ICARDA".</t>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Extract from the input text every CGIAR Initiative or Center only if it belongs to the Allowed Values list below. Ignore anything that is not in the list.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Allowed Values</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** CGIAR Centers (full name + acronym)
+Africa Rice Center (AfricaRice)
+Alliance of Bioversity and CIAT – Headquarter (Bioversity International) (ABC)
+Alliance of Bioversity and CIAT – Regional Hub (Centro Internacional de Agricultura Tropical) (ABC)
+Center for International Forestry Research (CIFOR)
+Centro Internacional de Mejoramiento de Maíz y Trigo (CIMMYT)
+Centro Internacional de la Papa (CIP)
+International Center for Agricultural Research in the Dry Areas (ICARDA)
+World Agroforestry Centre (ICRAF)
+International Crops Research Institute for the Semi-Arid Tropics (ICRISAT)
+International Food Policy Research Institute (IFPRI)
+International Institute of Tropical Agriculture (IITA)
+International Livestock Research Institute (ILRI)
+International Rice Research Institute (IRRI)
+International Water Management Institute (IWMI)
+WorldFish (WorldFish)
+System Organization (SO).
+Initiatives &amp; Platforms
+Accelerated Breeding
+Genebanks
+Breeding Resources
+Market Intelligence
+Seed Equal
+Protecting Human Health Through a One Health Approach
+One Health
+ActioNs for Innovative climate change Mitigation &amp; Adaptation of Livestock Systems (ANIMALS)
+ASPIRE – building integrated agrisilvopastoral food systems resilient to climate change and other crises
+From Fragility to Resilience in Central and West Asia and North Africa
+Fragility to Resilience in Central and West Asia and North Africa
+Excellence in Agronomy
+Nature-Positive Solutions
+Plant Health
+AgriLAC Resiliente
+Resilient Aquatic Food Systems for Healthy People and Planet
+Aquatic Foods
+Resilient Cities
+Sustainable Animal Productivity
+Asian Mega-Deltas
+Mixed Farming Systems
+Transforming Agrifood Systems in South Asia
+Ukama Ustawi: Diversification for Resilient Agrifood Systems in East and Southern Africa
+Diversification in East and Southern Africa
+Transforming AgriFood Systems in West and Central Africa
+West and Central African Food Systems Transformation
+ClimBeR: Building Systemic Resilience Against Climate Variability and Extremes
+Climate Resilience
+Foresight
+Digital Innovation
+Gender Equality
+National Policies and Strategies
+NEXUS Gains
+Rethinking Food Markets
+Sustainable Healthy Diets
+Agroecology
+Low-Emission Food Systems
+Fruit and Vegetables for Sustainable Healthy Diets
+Livestock and Climate
+Fragility, Conflict and Migration
+GENDER Impact Platform
+Climate Platform
+Environment and Biodiversity Impact Area Platform
+NUTRITION Impact Platform
+Genome Editing.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Output Format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Your response should be a string with values separated by commas. For example "CIMMYT, AgriLac Resiliente, ICARDA".</t>
     </r>
   </si>
   <si>
@@ -423,60 +507,69 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
       <t>**</t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Parameter:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Country of Study.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Description:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** The name of the country where the study/observations took place.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Reply with the name of the country, e.g. "Spain". If the study took place in more than one country, then list the different countries separated by commas, for example "Ghana, Ethiopia"</t>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Country of Study.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Description</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Extract only the explicitly named sovereign state(s) where the study or observations were carried out.
+• Accept a country only if it appears in the text as a clear, specific name (e.g. “Kenya”, “Ghana”).
+• Ignore vague, collective, or numeric references such as “several African countries”, “16 Asian nations”, “across Europe”, “LMICs”, etc.
+• If the study spans multiple specifically named countries, list every one.
+• If no specific country name is given, output None..
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Output Format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Reply with the name of the country, e.g. "Kenya". If the study took place in more than one country, then list the different countries separated by commas, for example "Ghana, Kenya"</t>
     </r>
   </si>
   <si>
@@ -723,7 +816,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>:** Crop/Product Type.
+      <t>:** Crop / Livestock / Technology.
 **</t>
     </r>
     <r>
@@ -741,25 +834,37 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>:** Identify the crop/product that is cover by CGIAR research in the impact study. By crop/product we are referring to a crop (e.g. cereals, legumes, fruits, and vegetables), livestock (e.g. cattle, poultry, fish, other animal species) or even an technology innovation. For crop and livestock your answer should be based on the vocabulary used in AGROVOC. It possible that CGIAR research is not link to a specific crop or livestock, when this is the case you should reply with "Not specific". And if you identifiy that CGIAR research is a technology you should reply "technology".
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Your response should be a string with the values separated by commas. Use your judgement and AGROVOC vocabulary for the response wording.</t>
+      <t>:**  
+Return the biological commodity (plant or animal species) that CGIAR research targets, **using the AGROVOC preferred label**.  
+Valid answers = crops (e.g. “rice”, “common bean”, “groundnut”) or livestock/aquatic species (e.g. “cattle”, “goat”, “Nile tilapia”).  
+Do **not** return:  
+ • Farming or management systems (e.g. “conservation agriculture”, “agroforestry”, “integrated pest management”).  
+ • Generic value-chain terms (e.g. “seed systems”, “marketing”).  
+ • Inputs (fertilizer, pesticide, irrigation).  
+ • Policies or socio-economic topics.  
+**Special cases**  
+• If the paper focuses on a **discrete technological innovation** (a tangible tool, piece of machinery, molecular-breeding method, digital platform, or software) *and* no single crop or livestock is central, return just "Technology". Broad agronomic approaches (e.g. “conservation agriculture”) are *not* “technology”.  
+• If no crop, livestock, or qualifying technology is clearly specified, return **“Not specific”**.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Output format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:**  
+A single string; if multiple valid species appear, list them alphabetically, separated by commas.  
+Example: "maize, rice, soybean"</t>
     </r>
   </si>
   <si>
@@ -892,12 +997,101 @@
 **Description:** Identify CGIAR research object. It could be a crop (e.g. cereals, legumes, fruits, and vegetables), livestock (e.g. cattle, poultry, fish, other animal species) or even an technology innovation. For crop your answer should be based on the vocabulary used in AGROVOC. It possible that CGIAR research is not link to a specific crop or livestock, when this is the case you should reply with "Not specific". And if you identifiy that CGIAR research object is a technology you should reply "technology".
 **Output Format:** Your response should be a string with the values separated by commas. Use your judgement and AGROVOC vocabulary for the response wording.</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Impact/Outcome Indicators
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Description</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">:** Identify mentions in the text of 
+1) Indicators used to assess the impact/outcome of CGIAR interventions,
+2) Units used to measure results, 
+3) The quantitative or qualitative results of the intervention. 
+Only capture these triplets if the numeric results are reported as statistically significant in the text. If multiple triplets are mentioned, output each as a list of three elements. For other significant or notable results (both quantitative or qualitative information that seems significant or relevant, although technically not statistically significant or not explicitly mentioned) capture them as a separate set of triples [Indicator, Units, Results]. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">You should start your analysis by screening the sections "Abstract" or "Conclusion" (or similar sections) and based on the findings  you could extend the search to other sections from the study to complete your search.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Output Format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** 
+- Return a list of lists, with each nested list containing exactly three items in the order: [Indicator, Units, Results].
+- Separate each nested list with a comma. 
+- If no valid triplets are found, return an empty list.
+- Example: `[[""Maize Yield"", ""%"", ""5% increase (p&lt;0.05)""], [""Adoption Rate"", ""Households"", ""20% adoption (p&lt;0.01)""]]`</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -941,6 +1135,12 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1218,16 +1418,16 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:N1"/>
-  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="21.59765625" customWidth="1"/>
-    <col min="5" max="5" width="21.59765625" customWidth="1"/>
-    <col min="7" max="7" width="71.59765625" customWidth="1"/>
-    <col min="8" max="9" width="21.59765625" customWidth="1"/>
-    <col min="14" max="14" width="21.59765625" customWidth="1"/>
+    <col min="1" max="2" width="21.5703125" customWidth="1"/>
+    <col min="5" max="6" width="21.5703125" customWidth="1"/>
+    <col min="7" max="8" width="71.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="338.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="338.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1243,13 +1443,13 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
@@ -1279,12 +1479,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E6D4E2-1D8F-48EE-9FAC-0B644E8606E1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.95"/>
   <cols>
-    <col min="1" max="1" width="89.8984375" customWidth="1"/>
+    <col min="1" max="1" width="89.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="104" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="104.1">
       <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
@@ -1292,4 +1492,22 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{458A5EEE-D46E-444F-BC25-E21054F1B9CE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="409.6">
+      <c r="A1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Final version approved by Hugo, working ready to process.
</commit_message>
<xml_diff>
--- a/questions_v3v2_June03.xlsx
+++ b/questions_v3v2_June03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/j_berenguer_cgiar_org/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F29851E9-F173-41FE-9B62-1FE3446C7755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8547FC0D-8979-4112-82E9-5998F00EDA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -479,7 +479,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** The CGIAR Impact Area(s) addresses by CGIAR intervention. The intervention should have/target at least one Impact Area. You should identify the primary and secondary CGIAR Impact Area(s) addresses by CGIAR intervention. Your analysis should be based on the CGIAR Impact Area(s) descriptions below.
+      <t>** You should identify the two main CGIAR Impact Areas addresses by the CGIAR intervention, the primary and secondary CGIAR Impact Area. Your analysis should be based on the CGIAR Impact Area(s) descriptions below.
 - (1) "Nutrition, health and food security": "Enable affordable, healthy diets for the 3 billion people who currently lack access to safe and nutritious food. Decrease cases of foodborne illness and zoonotic diseases by one-third."
 - (2) "Poverty reduction, livelihoods and jobs": "Lift at least 500 million people living in rural areas above the extreme poverty line of US $1.90 per day. Reduce by at least half the proportion of people of all ages living in poverty in all its dimensions."
 - (3) "Gender equality, youth and social inclusion": "Address disparities in rights to economic resources, ownership, and control over land and natural resources for women. Create opportunities for young people not in employment, education, or training, with a focus on gender inclusivity."
@@ -502,7 +502,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** Your response should be the primary and secondary CGIAR Impact Area with separated by commas. If the CGIAR intervention focuses only on one main Impact Area, then return the name of the Impact Area (from those above), without the description in this format: "Main Area Name; No Secondary Impact Area(s)". For example: "Climate adaptation and mitigation; No Secondary Impact Area(s)".</t>
+      <t>** Your response should be the primary and secondary CGIAR Impact Area with separated by commas (Max of 2 Impact Areas). If the CGIAR intervention focuses only on one main Impact Area, then return the name of the Impact Area (from those above), without the description in this format: "Main Area Name; No Secondary Impact Area(s)". For example: "Climate adaptation and mitigation; No Secondary Impact Area(s)".</t>
     </r>
   </si>
   <si>

</xml_diff>